<commit_message>
analysis: align Samyang RIM periods and refresh valuation output
</commit_message>
<xml_diff>
--- a/model/RIM_model.xlsx
+++ b/model/RIM_model.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rdceb89f3544446b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" r:id="R39372ef06dc04e43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Residual Income" sheetId="3" r:id="Rbdecefae807547da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="4" r:id="Rc7e0cfe1ca0647ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R15c1e214a3764247"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" r:id="Rff4d1b2814924c3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Residual Income" sheetId="3" r:id="R4fa4b21af7ed4d91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="4" r:id="Rfc8a87a166984969"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -553,7 +553,8 @@
         </x:is>
       </x:c>
       <x:c r="E4" s="4" t="n">
-        <x:v>837658.3163496589</x:v>
+        <x:f>'Residual Income'!B16</x:f>
+        <x:v>811036.4786541517</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -563,7 +564,8 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="5" t="n">
-        <x:v>6310.092661936726</x:v>
+        <x:f>'Residual Income'!B15</x:f>
+        <x:v>6109.549959248904</x:v>
       </x:c>
       <x:c r="C5" s="2" t="n"/>
       <x:c r="D5" s="3" t="inlineStr">
@@ -572,7 +574,8 @@
         </x:is>
       </x:c>
       <x:c r="E5" s="6" t="n">
-        <x:v>-0.3556474489618009</x:v>
+        <x:f>E4/E3-1</x:f>
+        <x:v>-0.3761257856506526</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -708,7 +711,7 @@
         <x:v>Provisional</x:v>
       </x:c>
       <x:c r="F4" s="3" t="str">
-        <x:v>2026H1 DART filing; consolidated equity. Reconcile to equity attributable to owners and NCI before treating as final common-equity base.</x:v>
+        <x:v>2026H1 consolidated equity proxy; reconcile parent-attributable equity and NCI before final per-share use</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -948,6 +951,85 @@
       <x:c r="D16" s="18"/>
       <x:c r="E16" s="18"/>
       <x:c r="F16" s="18"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>Period bridge</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>2026H1 reported net income</x:v>
+      </x:c>
+      <x:c r="C17" t="n">
+        <x:v>282.054</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>KRW bn</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>2026H1 consolidated net income</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>Period bridge</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>2026E full-year base net income</x:v>
+      </x:c>
+      <x:c r="C18" t="n">
+        <x:v>573.5</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>KRW bn</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>Analyst forecast</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>2026E Base scenario</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>Period bridge</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>2026H2 remaining net income</x:v>
+      </x:c>
+      <x:c r="C19" t="n">
+        <x:f>C18-C17</x:f>
+        <x:v>291.446</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>KRW bn</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>Formula</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>FY2026E Base less reported 2026H1 actual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>RIM method</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>Terminal RI formula</x:v>
+      </x:c>
+      <x:c r="C20"/>
+      <x:c r="D20" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>Method</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>BV2030 × (terminal ROE − CoE) × (1+g) / (CoE−g)</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1004,85 +1086,69 @@
       <x:c r="I2" s="2" t="n"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Year</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Beginning equity</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C3" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Net income</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D3" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Dividend</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E3" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Ending equity</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F3" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Equity charge</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G3" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Residual income</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H3" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">PV factor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I3" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">PV residual income</x:t>
-        </x:is>
+      <x:c r="A3" s="7" t="str">
+        <x:v>Period</x:v>
+      </x:c>
+      <x:c r="B3" s="7" t="str">
+        <x:v>Beginning equity</x:v>
+      </x:c>
+      <x:c r="C3" s="7" t="str">
+        <x:v>Net income</x:v>
+      </x:c>
+      <x:c r="D3" s="7" t="str">
+        <x:v>Dividend</x:v>
+      </x:c>
+      <x:c r="E3" s="7" t="str">
+        <x:v>Ending equity</x:v>
+      </x:c>
+      <x:c r="F3" s="7" t="str">
+        <x:v>Equity charge</x:v>
+      </x:c>
+      <x:c r="G3" s="7" t="str">
+        <x:v>Residual income</x:v>
+      </x:c>
+      <x:c r="H3" s="7" t="str">
+        <x:v>PV factor</x:v>
+      </x:c>
+      <x:c r="I3" s="7" t="str">
+        <x:v>PV residual income</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="3" t="n">
-        <x:v>2026</x:v>
+      <x:c r="A4" s="3" t="str">
+        <x:v>2026H2</x:v>
       </x:c>
       <x:c r="B4" s="5" t="n">
+        <x:f>Inputs!$C$4</x:f>
         <x:v>1548.3</x:v>
       </x:c>
       <x:c r="C4" s="5" t="n">
-        <x:v>573.5</x:v>
+        <x:f>Inputs!$C$19</x:f>
+        <x:v>291.446</x:v>
       </x:c>
       <x:c r="D4" s="5" t="n">
         <x:f>C4*Inputs!$C$7</x:f>
-        <x:v>86.02499999999999</x:v>
+        <x:v>43.7169</x:v>
       </x:c>
       <x:c r="E4" s="5" t="n">
         <x:f>B4+C4-D4</x:f>
-        <x:v>2035.775</x:v>
+        <x:v>1796.0291000000002</x:v>
       </x:c>
       <x:c r="F4" s="5" t="n">
-        <x:f>B4*Inputs!$C$6</x:f>
-        <x:v>139.34699999999998</x:v>
+        <x:f>B4*Inputs!$C$6*0.5</x:f>
+        <x:v>69.67349999999999</x:v>
       </x:c>
       <x:c r="G4" s="5" t="n">
         <x:f>C4-F4</x:f>
-        <x:v>434.153</x:v>
+        <x:v>221.77250000000004</x:v>
       </x:c>
       <x:c r="H4" s="8" t="n">
-        <x:f>1/(1+Inputs!$C$6)^(A4-2026+0.5)</x:f>
+        <x:f>1/(1+Inputs!$C$6)^0.5</x:f>
         <x:v>0.9578262852211513</x:v>
       </x:c>
       <x:c r="I4" s="5" t="n">
         <x:f>G4*H4</x:f>
-        <x:v>415.8431552076185</x:v>
+        <x:v>212.41952983920783</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1090,7 +1156,8 @@
         <x:v>2027</x:v>
       </x:c>
       <x:c r="B5" s="5" t="n">
-        <x:v>2035.775</x:v>
+        <x:f>E4</x:f>
+        <x:v>1796.0291000000002</x:v>
       </x:c>
       <x:c r="C5" s="5" t="n">
         <x:v>699.36</x:v>
@@ -1101,23 +1168,23 @@
       </x:c>
       <x:c r="E5" s="5" t="n">
         <x:f>B5+C5-D5</x:f>
-        <x:v>2630.231</x:v>
+        <x:v>2390.4851000000003</x:v>
       </x:c>
       <x:c r="F5" s="5" t="n">
         <x:f>B5*Inputs!$C$6</x:f>
-        <x:v>183.21975</x:v>
+        <x:v>161.64261900000002</x:v>
       </x:c>
       <x:c r="G5" s="5" t="n">
         <x:f>C5-F5</x:f>
-        <x:v>516.14025</x:v>
+        <x:v>537.7173809999999</x:v>
       </x:c>
       <x:c r="H5" s="8" t="n">
-        <x:f>1/(1+Inputs!$C$6)^(A5-2026+0.5)</x:f>
+        <x:f>1/(1+Inputs!$C$6)^1.5</x:f>
         <x:v>0.8787397112120654</x:v>
       </x:c>
       <x:c r="I5" s="5" t="n">
         <x:f>G5*H5</x:f>
-        <x:v>453.55293422992327</x:v>
+        <x:v>472.51361609364807</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1125,7 +1192,8 @@
         <x:v>2028</x:v>
       </x:c>
       <x:c r="B6" s="5" t="n">
-        <x:v>2630.231</x:v>
+        <x:f>E5</x:f>
+        <x:v>2390.4851000000003</x:v>
       </x:c>
       <x:c r="C6" s="5" t="n">
         <x:v>819.888</x:v>
@@ -1136,23 +1204,23 @@
       </x:c>
       <x:c r="E6" s="5" t="n">
         <x:f>B6+C6-D6</x:f>
-        <x:v>3327.1358</x:v>
+        <x:v>3087.3899</x:v>
       </x:c>
       <x:c r="F6" s="5" t="n">
         <x:f>B6*Inputs!$C$6</x:f>
-        <x:v>236.72079000000002</x:v>
+        <x:v>215.143659</x:v>
       </x:c>
       <x:c r="G6" s="5" t="n">
         <x:f>C6-F6</x:f>
-        <x:v>583.1672100000001</x:v>
+        <x:v>604.7443410000001</x:v>
       </x:c>
       <x:c r="H6" s="8" t="n">
-        <x:f>1/(1+Inputs!$C$6)^(A6-2026+0.5)</x:f>
+        <x:f>1/(1+Inputs!$C$6)^2.5</x:f>
         <x:v>0.8061832212954727</x:v>
       </x:c>
       <x:c r="I6" s="5" t="n">
         <x:f>G6*H6</x:f>
-        <x:v>470.13961991169344</x:v>
+        <x:v>487.5347408875879</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1160,7 +1228,8 @@
         <x:v>2029</x:v>
       </x:c>
       <x:c r="B7" s="5" t="n">
-        <x:v>3327.1358</x:v>
+        <x:f>E6</x:f>
+        <x:v>3087.3899</x:v>
       </x:c>
       <x:c r="C7" s="5" t="n">
         <x:v>903.775</x:v>
@@ -1171,23 +1240,23 @@
       </x:c>
       <x:c r="E7" s="5" t="n">
         <x:f>B7+C7-D7</x:f>
-        <x:v>4095.34455</x:v>
+        <x:v>3855.5986500000004</x:v>
       </x:c>
       <x:c r="F7" s="5" t="n">
         <x:f>B7*Inputs!$C$6</x:f>
-        <x:v>299.442222</x:v>
+        <x:v>277.865091</x:v>
       </x:c>
       <x:c r="G7" s="5" t="n">
         <x:f>C7-F7</x:f>
-        <x:v>604.332778</x:v>
+        <x:v>625.909909</x:v>
       </x:c>
       <x:c r="H7" s="8" t="n">
-        <x:f>1/(1+Inputs!$C$6)^(A7-2026+0.5)</x:f>
+        <x:f>1/(1+Inputs!$C$6)^3.5</x:f>
         <x:v>0.7396176342160301</x:v>
       </x:c>
       <x:c r="I7" s="5" t="n">
         <x:f>G7*H7</x:f>
-        <x:v>446.9751795435613</x:v>
+        <x:v>462.9340061269507</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1195,7 +1264,8 @@
         <x:v>2030</x:v>
       </x:c>
       <x:c r="B8" s="5" t="n">
-        <x:v>4095.34455</x:v>
+        <x:f>E7</x:f>
+        <x:v>3855.5986500000004</x:v>
       </x:c>
       <x:c r="C8" s="5" t="n">
         <x:v>969.311</x:v>
@@ -1206,23 +1276,93 @@
       </x:c>
       <x:c r="E8" s="5" t="n">
         <x:f>B8+C8-D8</x:f>
-        <x:v>4919.2589</x:v>
+        <x:v>4679.513000000001</x:v>
       </x:c>
       <x:c r="F8" s="5" t="n">
         <x:f>B8*Inputs!$C$6</x:f>
-        <x:v>368.5810095</x:v>
+        <x:v>347.00387850000004</x:v>
       </x:c>
       <x:c r="G8" s="5" t="n">
         <x:f>C8-F8</x:f>
-        <x:v>600.7299905</x:v>
+        <x:v>622.3071215</x:v>
       </x:c>
       <x:c r="H8" s="8" t="n">
-        <x:f>1/(1+Inputs!$C$6)^(A8-2026+0.5)</x:f>
+        <x:f>1/(1+Inputs!$C$6)^4.5</x:f>
         <x:v>0.6785482882715871</x:v>
       </x:c>
       <x:c r="I8" s="5" t="n">
         <x:f>G8*H8</x:f>
-        <x:v>407.62430676718174</x:v>
+        <x:v>422.26543207304354</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>RIM result</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>Starting equity</x:v>
+      </x:c>
+      <x:c r="B11" t="n">
+        <x:f>Inputs!$C$4</x:f>
+        <x:v>1548.3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>PV residual income</x:v>
+      </x:c>
+      <x:c r="B12" t="n">
+        <x:f>SUM(I4:I8)</x:f>
+        <x:v>2057.667325020438</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>Terminal RI value</x:v>
+      </x:c>
+      <x:c r="B13" t="n">
+        <x:f>E8*(Inputs!$C$8-Inputs!$C$6)*(1+Inputs!$C$9)/(Inputs!$C$6-Inputs!$C$9)</x:f>
+        <x:v>3689.6160192307702</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>PV terminal RI</x:v>
+      </x:c>
+      <x:c r="B14" t="n">
+        <x:f>B13/(1+Inputs!$C$6)^4.5</x:f>
+        <x:v>2503.5826342284663</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>RIM equity value</x:v>
+      </x:c>
+      <x:c r="B15" t="n">
+        <x:f>B11+B12+B14</x:f>
+        <x:v>6109.549959248904</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>Value per share</x:v>
+      </x:c>
+      <x:c r="B16" t="n">
+        <x:f>B15*1000/Inputs!$C$5</x:f>
+        <x:v>811036.4786541517</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>Terminal RI uses next-period growth</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>TV uses RI_(t+1); growth factor is included</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1293,13 +1433,13 @@
         <x:v>0.08</x:v>
       </x:c>
       <x:c r="B4" s="4" t="n">
-        <x:v>853982.7778084386</x:v>
+        <x:v>825597.0298841606</x:v>
       </x:c>
       <x:c r="C4" s="4" t="n">
-        <x:v>1021937.126951786</x:v>
+        <x:v>989360.1475823164</x:v>
       </x:c>
       <x:c r="D4" s="4" t="n">
-        <x:v>1189891.476095132</x:v>
+        <x:v>1153123.265280472</x:v>
       </x:c>
       <x:c r="E4" s="2" t="n"/>
       <x:c r="F4" s="2" t="n"/>
@@ -1309,13 +1449,13 @@
         <x:v>0.08500000000000001</x:v>
       </x:c>
       <x:c r="B5" s="4" t="n">
-        <x:v>771196.6618216623</x:v>
+        <x:v>745558.813937585</x:v>
       </x:c>
       <x:c r="C5" s="4" t="n">
-        <x:v>921987.7833215365</x:v>
+        <x:v>892587.0052525045</x:v>
       </x:c>
       <x:c r="D5" s="4" t="n">
-        <x:v>1072778.90482141</x:v>
+        <x:v>1039615.1965674239</x:v>
       </x:c>
       <x:c r="E5" s="2" t="n"/>
       <x:c r="F5" s="2" t="n"/>
@@ -1325,13 +1465,13 @@
         <x:v>0.09</x:v>
       </x:c>
       <x:c r="B6" s="4" t="n">
-        <x:v>701316.7603444339</x:v>
+        <x:v>678097.2698922699</x:v>
       </x:c>
       <x:c r="C6" s="4" t="n">
-        <x:v>837658.3163496589</x:v>
+        <x:v>811036.4786541517</x:v>
       </x:c>
       <x:c r="D6" s="4" t="n">
-        <x:v>973999.8723548837</x:v>
+        <x:v>943975.6874160332</x:v>
       </x:c>
       <x:c r="E6" s="2" t="n"/>
       <x:c r="F6" s="2" t="n"/>
@@ -1341,13 +1481,13 @@
         <x:v>0.095</x:v>
       </x:c>
       <x:c r="B7" s="4" t="n">
-        <x:v>641571.0550625738</x:v>
+        <x:v>620509.7334736735</x:v>
       </x:c>
       <x:c r="C7" s="4" t="n">
-        <x:v>765593.208298385</x:v>
+        <x:v>741436.9650763536</x:v>
       </x:c>
       <x:c r="D7" s="4" t="n">
-        <x:v>889615.3615341963</x:v>
+        <x:v>862364.1966790337</x:v>
       </x:c>
       <x:c r="E7" s="2" t="n"/>
       <x:c r="F7" s="2" t="n"/>
@@ -1357,13 +1497,13 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="B8" s="4" t="n">
-        <x:v>589926.9388832611</x:v>
+        <x:v>570814.4942494262</x:v>
       </x:c>
       <x:c r="C8" s="4" t="n">
-        <x:v>703332.0156408824</x:v>
+        <x:v>681389.5941343133</x:v>
       </x:c>
       <x:c r="D8" s="4" t="n">
-        <x:v>816737.0923985039</x:v>
+        <x:v>791964.6940192003</x:v>
       </x:c>
       <x:c r="E8" s="2" t="n"/>
       <x:c r="F8" s="2" t="n"/>

</xml_diff>